<commit_message>
Sum Diff in GC per entity netting file
</commit_message>
<xml_diff>
--- a/outputs/entities/FX-Netting-L_4016_DE-2026-08-24.xlsx
+++ b/outputs/entities/FX-Netting-L_4016_DE-2026-08-24.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Netting" sheetId="1" r:id="R0e9580aee92b47df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Details" sheetId="2" r:id="R5d94ed6238b9474f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Netting" sheetId="1" r:id="Rd9e6656b78c04ef5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Details" sheetId="2" r:id="R1586ae9ba6e446e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -301,7 +301,6 @@
     <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -313,18 +312,16 @@
       <x:c r="D1" s="2"/>
       <x:c r="E1" s="2"/>
       <x:c r="F1" s="2"/>
-      <x:c r="G1" s="2"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="str">
-        <x:v>Summierung der FX-Geschäfte | Quelle: GitHub Issue #2 | 1 Geschäfte</x:v>
+        <x:v>Summierung von „Diff. in GC“ | Quelle: GitHub Issue #2 | 1 Geschäfte</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
       <x:c r="D2" s="4"/>
       <x:c r="E2" s="4"/>
       <x:c r="F2" s="4"/>
-      <x:c r="G2" s="4"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="6" t="str">
@@ -343,10 +340,7 @@
         <x:v>Deals</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Net Amount</x:v>
-      </x:c>
-      <x:c r="G4" s="6" t="str">
-        <x:v>Net EUR Equivalent</x:v>
+        <x:v>Sum Diff. in GC</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -367,18 +361,14 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:f>SUMIFS('Details'!$I$2:$I$2,'Details'!$B$2:$B$2,A5,'Details'!$C$2:$C$2,B5,'Details'!$E$2:$E$2,C5,'Details'!$H$2:$H$2,D5)</x:f>
-        <x:v>300000</x:v>
-      </x:c>
-      <x:c r="G5" s="9" t="n">
-        <x:f>SUMIFS('Details'!$L$2:$L$2,'Details'!$B$2:$B$2,A5,'Details'!$C$2:$C$2,B5,'Details'!$E$2:$E$2,C5,'Details'!$H$2:$H$2,D5)</x:f>
-        <x:v>-203307.13</x:v>
+        <x:f>SUMIFS('Details'!$N$2:$N$2,'Details'!$B$2:$B$2,A5,'Details'!$C$2:$C$2,B5,'Details'!$E$2:$E$2,C5,'Details'!$H$2:$H$2,D5)</x:f>
+        <x:v>-1422.88</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:G1"/>
-    <x:mergeCell ref="A2:G2"/>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Format and total Diff in GC by entity
</commit_message>
<xml_diff>
--- a/outputs/entities/FX-Netting-L_4016_DE-2026-08-24.xlsx
+++ b/outputs/entities/FX-Netting-L_4016_DE-2026-08-24.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Netting" sheetId="1" r:id="Rd9e6656b78c04ef5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Details" sheetId="2" r:id="R1586ae9ba6e446e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Netting" sheetId="1" r:id="R31d8ceedfd384f78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Details" sheetId="2" r:id="R6098d59d964447b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,10 +16,10 @@
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
-    <x:numFmt numFmtId="201" formatCode="#,##0.00;[Red](#,##0.00);-"/>
+    <x:numFmt numFmtId="201" formatCode="#,##0.00;[Red]-#,##0.00;-"/>
     <x:numFmt numFmtId="202" formatCode="0.0000"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -39,6 +39,11 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -65,13 +70,18 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="2">
     <x:border/>
+    <x:border>
+      <x:top style="medium">
+        <x:color rgb="FF17365D"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -84,6 +94,9 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -365,10 +378,24 @@
         <x:v>-1422.88</x:v>
       </x:c>
     </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="str">
+        <x:v>Summe Diff. in GC</x:v>
+      </x:c>
+      <x:c r="B6" s="11"/>
+      <x:c r="C6" s="11"/>
+      <x:c r="D6" s="11"/>
+      <x:c r="E6" s="11"/>
+      <x:c r="F6" s="12" t="n">
+        <x:f>SUM(F5:F5)</x:f>
+        <x:v>-1422.88</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
     <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A6:E6"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -397,52 +424,52 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="13" t="str">
+      <x:c r="A1" s="16" t="str">
         <x:v>Reference</x:v>
       </x:c>
-      <x:c r="B1" s="13" t="str">
+      <x:c r="B1" s="16" t="str">
         <x:v>Entity</x:v>
       </x:c>
-      <x:c r="C1" s="13" t="str">
+      <x:c r="C1" s="16" t="str">
         <x:v>Counterparty</x:v>
       </x:c>
-      <x:c r="D1" s="13" t="str">
+      <x:c r="D1" s="16" t="str">
         <x:v>Int/Ext</x:v>
       </x:c>
-      <x:c r="E1" s="13" t="str">
+      <x:c r="E1" s="16" t="str">
         <x:v>Value Date</x:v>
       </x:c>
-      <x:c r="F1" s="13" t="str">
+      <x:c r="F1" s="16" t="str">
         <x:v>Deal Type</x:v>
       </x:c>
-      <x:c r="G1" s="13" t="str">
+      <x:c r="G1" s="16" t="str">
         <x:v>Buy/Sell</x:v>
       </x:c>
-      <x:c r="H1" s="13" t="str">
+      <x:c r="H1" s="16" t="str">
         <x:v>Currency</x:v>
       </x:c>
-      <x:c r="I1" s="13" t="str">
+      <x:c r="I1" s="16" t="str">
         <x:v>Amount</x:v>
       </x:c>
-      <x:c r="J1" s="13" t="str">
+      <x:c r="J1" s="16" t="str">
         <x:v>Rate</x:v>
       </x:c>
-      <x:c r="K1" s="13" t="str">
+      <x:c r="K1" s="16" t="str">
         <x:v>Equivalent Currency</x:v>
       </x:c>
-      <x:c r="L1" s="13" t="str">
+      <x:c r="L1" s="16" t="str">
         <x:v>Equivalent Amount EUR</x:v>
       </x:c>
-      <x:c r="M1" s="13" t="str">
+      <x:c r="M1" s="16" t="str">
         <x:v>Mark-to-market</x:v>
       </x:c>
-      <x:c r="N1" s="13" t="str">
+      <x:c r="N1" s="16" t="str">
         <x:v>Diff. in GC</x:v>
       </x:c>
-      <x:c r="O1" s="13" t="str">
+      <x:c r="O1" s="16" t="str">
         <x:v>Amount (MTM) EUR</x:v>
       </x:c>
-      <x:c r="P1" s="13" t="str">
+      <x:c r="P1" s="16" t="str">
         <x:v>Portfolio</x:v>
       </x:c>
     </x:row>
@@ -474,7 +501,7 @@
       <x:c r="I2" s="9" t="n">
         <x:v>300000</x:v>
       </x:c>
-      <x:c r="J2" s="14" t="n">
+      <x:c r="J2" s="17" t="n">
         <x:v>1.4756</x:v>
       </x:c>
       <x:c r="K2" t="str">

</xml_diff>